<commit_message>
Add Code.gs + Google Sheets sync for Aktien/Trades
- Code.gs: vollständiger Apps-Script-Code direkt in der App anzeigbar
  und per Knopfdruck in die Zwischenablage kopierbar (Setup Schritt 2)
- Aktien & Trades werden bei bestehender Sheet-Verbindung in Google
  Sheets gespeichert (Sheets: 'Aktien' A–F, 'Trades' A–J)
- loadAll() lädt Aktien/Trades aus Sheets (fallback auf localStorage)
- saveNewAktie / saveTrade / deleteTrade / deleteAktie synchen live
- Excel-Template: neue Sheets 'Aktien' und 'Trades' mit Swissquote-
  Beispieldaten und Ticker-Hinweisen (ZURN.SW, IQQE.DE, SAAB-B.ST …)

https://claude.ai/code/session_01BknN7Dny1eVCqQo34UDGL4
</commit_message>
<xml_diff>
--- a/finanztracker_template.xlsx
+++ b/finanztracker_template.xlsx
@@ -12,7 +12,9 @@
     <sheet name="Einnahmen" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="Daueraufträge" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="Kategorien" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Einstellungen" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Aktien" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Trades" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Einstellungen" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -753,7 +755,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B34"/>
+  <dimension ref="A1:B42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="74" customWidth="1" min="1" max="1"/>
@@ -879,7 +881,7 @@
     <row r="21" ht="16" customHeight="1">
       <c r="A21" s="3" t="inlineStr">
         <is>
-          <t>⚠  Tabellenblattnamen (Ausgaben, Einnahmen, Daueraufträge, Kategorien, Einstellungen) nicht umbenennen.</t>
+          <t>⚠  Tabellenblattnamen (Ausgaben, Einnahmen, Daueraufträge, Kategorien, Einstellungen, Aktien, Trades) nicht umbenennen.</t>
         </is>
       </c>
     </row>
@@ -901,14 +903,14 @@
     <row r="25" ht="16" customHeight="1">
       <c r="A25" s="3" t="inlineStr">
         <is>
-          <t>Ausgaben:      ID | Datum | Beschreibung | Kategorie | Betrag | Notiz | Deleted</t>
+          <t>Ausgaben:      ID | Datum | Beschreibung | Kategorie | Betrag | Notiz | Deleted | isFixkosten</t>
         </is>
       </c>
     </row>
     <row r="26" ht="16" customHeight="1">
       <c r="A26" s="3" t="inlineStr">
         <is>
-          <t>Einnahmen:     ID | Datum | Beschreibung | Kategorie | Betrag | Notiz | Deleted</t>
+          <t>Einnahmen:     ID | Datum | Beschreibung | Kategorie | Betrag | Notiz | Deleted | isLohn</t>
         </is>
       </c>
     </row>
@@ -933,32 +935,82 @@
         </is>
       </c>
     </row>
-    <row r="30" ht="8" customHeight="1"/>
-    <row r="31" ht="20" customHeight="1">
-      <c r="A31" s="2" t="inlineStr">
+    <row r="30" ht="16" customHeight="1">
+      <c r="A30" s="3" t="inlineStr">
+        <is>
+          <t>Aktien:        ID | Titel | ISIN | Ticker (Yahoo Finance) | Währung | Deleted</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="16" customHeight="1">
+      <c r="A31" s="3" t="inlineStr">
+        <is>
+          <t>Trades:        ID | AktieID | Typ (kauf/verkauf) | Datum | Anzahl | Preis/Stk | Währung | Courtage | Gesamt | Deleted</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="8" customHeight="1"/>
+    <row r="33" ht="20" customHeight="1">
+      <c r="A33" s="2" t="inlineStr">
         <is>
           <t>Kategorien anpassen</t>
-        </is>
-      </c>
-    </row>
-    <row r="32" ht="16" customHeight="1">
-      <c r="A32" s="3" t="inlineStr">
-        <is>
-          <t>→  Im Sheet 'Kategorien' beliebige Zeilen hinzufügen/ändern.</t>
-        </is>
-      </c>
-    </row>
-    <row r="33" ht="16" customHeight="1">
-      <c r="A33" s="3" t="inlineStr">
-        <is>
-          <t>→  Typ muss exakt 'ausgabe' oder 'einnahme' sein.</t>
         </is>
       </c>
     </row>
     <row r="34" ht="16" customHeight="1">
       <c r="A34" s="3" t="inlineStr">
         <is>
+          <t>→  Im Sheet 'Kategorien' beliebige Zeilen hinzufügen/ändern.</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" ht="16" customHeight="1">
+      <c r="A35" s="3" t="inlineStr">
+        <is>
+          <t>→  Typ muss exakt 'ausgabe' oder 'einnahme' sein.</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="16" customHeight="1">
+      <c r="A36" s="3" t="inlineStr">
+        <is>
           <t>→  Farbe: Hex-Code mit # z.B. #FF6B35</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" ht="8" customHeight="1"/>
+    <row r="38" ht="20" customHeight="1">
+      <c r="A38" s="2" t="inlineStr">
+        <is>
+          <t>Aktien-Ticker (Yahoo Finance Symbole)</t>
+        </is>
+      </c>
+    </row>
+    <row r="39" ht="16" customHeight="1">
+      <c r="A39" s="3" t="inlineStr">
+        <is>
+          <t>→  Schweizer Aktien:  ZURN.SW, ABBN.SW, NESN.SW, UBSG.SW  (Suffix .SW)</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" ht="16" customHeight="1">
+      <c r="A40" s="3" t="inlineStr">
+        <is>
+          <t>→  ETFs auf XETRA:   IQQE.DE, CSSMI.SW  (Suffix .DE oder .SW)</t>
+        </is>
+      </c>
+    </row>
+    <row r="41" ht="16" customHeight="1">
+      <c r="A41" s="3" t="inlineStr">
+        <is>
+          <t>→  Schwedische Aktien: SAAB-B.ST  (Suffix .ST)</t>
+        </is>
+      </c>
+    </row>
+    <row r="42" ht="16" customHeight="1">
+      <c r="A42" s="3" t="inlineStr">
+        <is>
+          <t>→  US-Aktien:         AAPL, MSFT  (kein Suffix)</t>
         </is>
       </c>
     </row>
@@ -2153,6 +2205,962 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
+    <tabColor rgb="00F7C948"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F13"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="16" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="10" customWidth="1" min="5" max="5"/>
+    <col width="9" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="20" customHeight="1">
+      <c r="A1" s="4" t="inlineStr">
+        <is>
+          <t>ID</t>
+        </is>
+      </c>
+      <c r="B1" s="4" t="inlineStr">
+        <is>
+          <t>Titel</t>
+        </is>
+      </c>
+      <c r="C1" s="4" t="inlineStr">
+        <is>
+          <t>ISIN</t>
+        </is>
+      </c>
+      <c r="D1" s="4" t="inlineStr">
+        <is>
+          <t>Ticker (Yahoo)</t>
+        </is>
+      </c>
+      <c r="E1" s="4" t="inlineStr">
+        <is>
+          <t>Währung</t>
+        </is>
+      </c>
+      <c r="F1" s="4" t="inlineStr">
+        <is>
+          <t>Deleted</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="5" t="inlineStr">
+        <is>
+          <t>st_001</t>
+        </is>
+      </c>
+      <c r="B2" s="5" t="inlineStr">
+        <is>
+          <t>Zurich Insurance N</t>
+        </is>
+      </c>
+      <c r="C2" s="5" t="inlineStr">
+        <is>
+          <t>CH0011075394</t>
+        </is>
+      </c>
+      <c r="D2" s="5" t="inlineStr">
+        <is>
+          <t>ZURN.SW</t>
+        </is>
+      </c>
+      <c r="E2" s="5" t="inlineStr">
+        <is>
+          <t>CHF</t>
+        </is>
+      </c>
+      <c r="F2" s="5" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="6" t="inlineStr">
+        <is>
+          <t>st_002</t>
+        </is>
+      </c>
+      <c r="B3" s="6" t="inlineStr">
+        <is>
+          <t>iSh EURSTx50 DE EUR D</t>
+        </is>
+      </c>
+      <c r="C3" s="6" t="inlineStr">
+        <is>
+          <t>DE0005933956</t>
+        </is>
+      </c>
+      <c r="D3" s="6" t="inlineStr">
+        <is>
+          <t>IQQE.DE</t>
+        </is>
+      </c>
+      <c r="E3" s="6" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="F3" s="6" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>st_003</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="inlineStr">
+        <is>
+          <t>iSh SLI CH CHF D</t>
+        </is>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>CH0031768937</t>
+        </is>
+      </c>
+      <c r="D4" s="5" t="inlineStr">
+        <is>
+          <t>CSSLI.SW</t>
+        </is>
+      </c>
+      <c r="E4" s="5" t="inlineStr">
+        <is>
+          <t>CHF</t>
+        </is>
+      </c>
+      <c r="F4" s="5" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="6" t="inlineStr">
+        <is>
+          <t>st_004</t>
+        </is>
+      </c>
+      <c r="B5" s="6" t="inlineStr">
+        <is>
+          <t>UBSETF SMI CHF DIS</t>
+        </is>
+      </c>
+      <c r="C5" s="6" t="inlineStr">
+        <is>
+          <t>CH0017142719</t>
+        </is>
+      </c>
+      <c r="D5" s="6" t="inlineStr">
+        <is>
+          <t>CSSMI.SW</t>
+        </is>
+      </c>
+      <c r="E5" s="6" t="inlineStr">
+        <is>
+          <t>CHF</t>
+        </is>
+      </c>
+      <c r="F5" s="6" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>st_005</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>Nestlé N</t>
+        </is>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>CH0038863350</t>
+        </is>
+      </c>
+      <c r="D6" s="5" t="inlineStr">
+        <is>
+          <t>NESN.SW</t>
+        </is>
+      </c>
+      <c r="E6" s="5" t="inlineStr">
+        <is>
+          <t>CHF</t>
+        </is>
+      </c>
+      <c r="F6" s="5" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="6" t="inlineStr">
+        <is>
+          <t>st_006</t>
+        </is>
+      </c>
+      <c r="B7" s="6" t="inlineStr">
+        <is>
+          <t>UBS Group N</t>
+        </is>
+      </c>
+      <c r="C7" s="6" t="inlineStr">
+        <is>
+          <t>CH0244767585</t>
+        </is>
+      </c>
+      <c r="D7" s="6" t="inlineStr">
+        <is>
+          <t>UBSG.SW</t>
+        </is>
+      </c>
+      <c r="E7" s="6" t="inlineStr">
+        <is>
+          <t>CHF</t>
+        </is>
+      </c>
+      <c r="F7" s="6" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>st_007</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="inlineStr">
+        <is>
+          <t>UBS Sol. China Tech UCITS USD</t>
+        </is>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>LU2265794276</t>
+        </is>
+      </c>
+      <c r="D8" s="5" t="inlineStr">
+        <is>
+          <t>UBCT.SW</t>
+        </is>
+      </c>
+      <c r="E8" s="5" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="F8" s="5" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="6" t="inlineStr">
+        <is>
+          <t>st_008</t>
+        </is>
+      </c>
+      <c r="B9" s="6" t="inlineStr">
+        <is>
+          <t>SAAB ORD</t>
+        </is>
+      </c>
+      <c r="C9" s="6" t="inlineStr">
+        <is>
+          <t>SE0021921269</t>
+        </is>
+      </c>
+      <c r="D9" s="6" t="inlineStr">
+        <is>
+          <t>SAAB-B.ST</t>
+        </is>
+      </c>
+      <c r="E9" s="6" t="inlineStr">
+        <is>
+          <t>SEK</t>
+        </is>
+      </c>
+      <c r="F9" s="6" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>st_009</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="inlineStr">
+        <is>
+          <t>ABB Ltd N</t>
+        </is>
+      </c>
+      <c r="C10" s="5" t="inlineStr"/>
+      <c r="D10" s="5" t="inlineStr">
+        <is>
+          <t>ABBN.SW</t>
+        </is>
+      </c>
+      <c r="E10" s="5" t="inlineStr">
+        <is>
+          <t>CHF</t>
+        </is>
+      </c>
+      <c r="F10" s="5" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="7" t="inlineStr">
+        <is>
+          <t>Ticker-Beispiele: .SW = Schweiz, .DE = XETRA, .ST = Stockholm, kein Suffix = USA</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <tabColor rgb="0056B6C2"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:J18"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="16" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="9" customWidth="1" min="3" max="3"/>
+    <col width="13" customWidth="1" min="4" max="4"/>
+    <col width="10" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="10" customWidth="1" min="7" max="7"/>
+    <col width="10" customWidth="1" min="8" max="8"/>
+    <col width="14" customWidth="1" min="9" max="9"/>
+    <col width="9" customWidth="1" min="10" max="10"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="20" customHeight="1">
+      <c r="A1" s="4" t="inlineStr">
+        <is>
+          <t>ID</t>
+        </is>
+      </c>
+      <c r="B1" s="4" t="inlineStr">
+        <is>
+          <t>AktieID</t>
+        </is>
+      </c>
+      <c r="C1" s="4" t="inlineStr">
+        <is>
+          <t>Typ</t>
+        </is>
+      </c>
+      <c r="D1" s="4" t="inlineStr">
+        <is>
+          <t>Datum</t>
+        </is>
+      </c>
+      <c r="E1" s="4" t="inlineStr">
+        <is>
+          <t>Anzahl</t>
+        </is>
+      </c>
+      <c r="F1" s="4" t="inlineStr">
+        <is>
+          <t>Preis/Stk</t>
+        </is>
+      </c>
+      <c r="G1" s="4" t="inlineStr">
+        <is>
+          <t>Währung</t>
+        </is>
+      </c>
+      <c r="H1" s="4" t="inlineStr">
+        <is>
+          <t>Courtage</t>
+        </is>
+      </c>
+      <c r="I1" s="4" t="inlineStr">
+        <is>
+          <t>Gesamt</t>
+        </is>
+      </c>
+      <c r="J1" s="4" t="inlineStr">
+        <is>
+          <t>Deleted</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="5" t="inlineStr">
+        <is>
+          <t>tr_001</t>
+        </is>
+      </c>
+      <c r="B2" s="5" t="inlineStr">
+        <is>
+          <t>st_001</t>
+        </is>
+      </c>
+      <c r="C2" s="5" t="inlineStr">
+        <is>
+          <t>kauf</t>
+        </is>
+      </c>
+      <c r="D2" s="5" t="inlineStr">
+        <is>
+          <t>2025-04-02</t>
+        </is>
+      </c>
+      <c r="E2" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="F2" s="5" t="n">
+        <v>622</v>
+      </c>
+      <c r="G2" s="5" t="inlineStr">
+        <is>
+          <t>CHF</t>
+        </is>
+      </c>
+      <c r="H2" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="I2" s="5" t="n">
+        <v>2488</v>
+      </c>
+      <c r="J2" s="5" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="6" t="inlineStr">
+        <is>
+          <t>tr_002</t>
+        </is>
+      </c>
+      <c r="B3" s="6" t="inlineStr">
+        <is>
+          <t>st_001</t>
+        </is>
+      </c>
+      <c r="C3" s="6" t="inlineStr">
+        <is>
+          <t>verkauf</t>
+        </is>
+      </c>
+      <c r="D3" s="6" t="inlineStr">
+        <is>
+          <t>2025-10-03</t>
+        </is>
+      </c>
+      <c r="E3" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="F3" s="6" t="n">
+        <v>571.2</v>
+      </c>
+      <c r="G3" s="6" t="inlineStr">
+        <is>
+          <t>CHF</t>
+        </is>
+      </c>
+      <c r="H3" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="I3" s="6" t="n">
+        <v>1142.4</v>
+      </c>
+      <c r="J3" s="6" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>tr_003</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="inlineStr">
+        <is>
+          <t>st_002</t>
+        </is>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>kauf</t>
+        </is>
+      </c>
+      <c r="D4" s="5" t="inlineStr">
+        <is>
+          <t>2025-04-11</t>
+        </is>
+      </c>
+      <c r="E4" s="5" t="n">
+        <v>31</v>
+      </c>
+      <c r="F4" s="5" t="n">
+        <v>47.915</v>
+      </c>
+      <c r="G4" s="5" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="H4" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="I4" s="5" t="n">
+        <v>1485.37</v>
+      </c>
+      <c r="J4" s="5" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="6" t="inlineStr">
+        <is>
+          <t>tr_004</t>
+        </is>
+      </c>
+      <c r="B5" s="6" t="inlineStr">
+        <is>
+          <t>st_002</t>
+        </is>
+      </c>
+      <c r="C5" s="6" t="inlineStr">
+        <is>
+          <t>verkauf</t>
+        </is>
+      </c>
+      <c r="D5" s="6" t="inlineStr">
+        <is>
+          <t>2025-04-09</t>
+        </is>
+      </c>
+      <c r="E5" s="6" t="n">
+        <v>18</v>
+      </c>
+      <c r="F5" s="6" t="n">
+        <v>54.5</v>
+      </c>
+      <c r="G5" s="6" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="H5" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="I5" s="6" t="n">
+        <v>981</v>
+      </c>
+      <c r="J5" s="6" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>tr_005</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>st_003</t>
+        </is>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>kauf</t>
+        </is>
+      </c>
+      <c r="D6" s="5" t="inlineStr">
+        <is>
+          <t>2025-04-10</t>
+        </is>
+      </c>
+      <c r="E6" s="5" t="n">
+        <v>8</v>
+      </c>
+      <c r="F6" s="5" t="n">
+        <v>193.4</v>
+      </c>
+      <c r="G6" s="5" t="inlineStr">
+        <is>
+          <t>CHF</t>
+        </is>
+      </c>
+      <c r="H6" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="I6" s="5" t="n">
+        <v>1547.2</v>
+      </c>
+      <c r="J6" s="5" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="6" t="inlineStr">
+        <is>
+          <t>tr_006</t>
+        </is>
+      </c>
+      <c r="B7" s="6" t="inlineStr">
+        <is>
+          <t>st_003</t>
+        </is>
+      </c>
+      <c r="C7" s="6" t="inlineStr">
+        <is>
+          <t>verkauf</t>
+        </is>
+      </c>
+      <c r="D7" s="6" t="inlineStr">
+        <is>
+          <t>2025-10-03</t>
+        </is>
+      </c>
+      <c r="E7" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="F7" s="6" t="n">
+        <v>214.55</v>
+      </c>
+      <c r="G7" s="6" t="inlineStr">
+        <is>
+          <t>CHF</t>
+        </is>
+      </c>
+      <c r="H7" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="I7" s="6" t="n">
+        <v>429.1</v>
+      </c>
+      <c r="J7" s="6" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>tr_007</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="inlineStr">
+        <is>
+          <t>st_004</t>
+        </is>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>kauf</t>
+        </is>
+      </c>
+      <c r="D8" s="5" t="inlineStr">
+        <is>
+          <t>2025-04-09</t>
+        </is>
+      </c>
+      <c r="E8" s="5" t="n">
+        <v>10</v>
+      </c>
+      <c r="F8" s="5" t="n">
+        <v>112.2</v>
+      </c>
+      <c r="G8" s="5" t="inlineStr">
+        <is>
+          <t>CHF</t>
+        </is>
+      </c>
+      <c r="H8" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="I8" s="5" t="n">
+        <v>1122</v>
+      </c>
+      <c r="J8" s="5" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="6" t="inlineStr">
+        <is>
+          <t>tr_008</t>
+        </is>
+      </c>
+      <c r="B9" s="6" t="inlineStr">
+        <is>
+          <t>st_004</t>
+        </is>
+      </c>
+      <c r="C9" s="6" t="inlineStr">
+        <is>
+          <t>verkauf</t>
+        </is>
+      </c>
+      <c r="D9" s="6" t="inlineStr">
+        <is>
+          <t>2025-12-16</t>
+        </is>
+      </c>
+      <c r="E9" s="6" t="n">
+        <v>10</v>
+      </c>
+      <c r="F9" s="6" t="n">
+        <v>1316.95</v>
+      </c>
+      <c r="G9" s="6" t="inlineStr">
+        <is>
+          <t>CHF</t>
+        </is>
+      </c>
+      <c r="H9" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="I9" s="6" t="n">
+        <v>13169.5</v>
+      </c>
+      <c r="J9" s="6" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>tr_009</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="inlineStr">
+        <is>
+          <t>st_005</t>
+        </is>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>kauf</t>
+        </is>
+      </c>
+      <c r="D10" s="5" t="inlineStr">
+        <is>
+          <t>2025-04-02</t>
+        </is>
+      </c>
+      <c r="E10" s="5" t="n">
+        <v>22</v>
+      </c>
+      <c r="F10" s="5" t="n">
+        <v>90</v>
+      </c>
+      <c r="G10" s="5" t="inlineStr">
+        <is>
+          <t>CHF</t>
+        </is>
+      </c>
+      <c r="H10" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="I10" s="5" t="n">
+        <v>1980</v>
+      </c>
+      <c r="J10" s="5" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="6" t="inlineStr">
+        <is>
+          <t>tr_010</t>
+        </is>
+      </c>
+      <c r="B11" s="6" t="inlineStr">
+        <is>
+          <t>st_006</t>
+        </is>
+      </c>
+      <c r="C11" s="6" t="inlineStr">
+        <is>
+          <t>kauf</t>
+        </is>
+      </c>
+      <c r="D11" s="6" t="inlineStr">
+        <is>
+          <t>2025-04-29</t>
+        </is>
+      </c>
+      <c r="E11" s="6" t="n">
+        <v>25</v>
+      </c>
+      <c r="F11" s="6" t="n">
+        <v>43</v>
+      </c>
+      <c r="G11" s="6" t="inlineStr">
+        <is>
+          <t>CHF</t>
+        </is>
+      </c>
+      <c r="H11" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="I11" s="6" t="n">
+        <v>1075</v>
+      </c>
+      <c r="J11" s="6" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="5" t="inlineStr">
+        <is>
+          <t>tr_011</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="inlineStr">
+        <is>
+          <t>st_006</t>
+        </is>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>verkauf</t>
+        </is>
+      </c>
+      <c r="D12" s="5" t="inlineStr">
+        <is>
+          <t>2025-09-04</t>
+        </is>
+      </c>
+      <c r="E12" s="5" t="n">
+        <v>15</v>
+      </c>
+      <c r="F12" s="5" t="n">
+        <v>32.3</v>
+      </c>
+      <c r="G12" s="5" t="inlineStr">
+        <is>
+          <t>CHF</t>
+        </is>
+      </c>
+      <c r="H12" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="I12" s="5" t="n">
+        <v>484.5</v>
+      </c>
+      <c r="J12" s="5" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="6" t="inlineStr">
+        <is>
+          <t>tr_012</t>
+        </is>
+      </c>
+      <c r="B13" s="6" t="inlineStr">
+        <is>
+          <t>st_007</t>
+        </is>
+      </c>
+      <c r="C13" s="6" t="inlineStr">
+        <is>
+          <t>kauf</t>
+        </is>
+      </c>
+      <c r="D13" s="6" t="inlineStr">
+        <is>
+          <t>2025-09-11</t>
+        </is>
+      </c>
+      <c r="E13" s="6" t="n">
+        <v>176</v>
+      </c>
+      <c r="F13" s="6" t="n">
+        <v>9.199999999999999</v>
+      </c>
+      <c r="G13" s="6" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="H13" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="I13" s="6" t="n">
+        <v>1619.2</v>
+      </c>
+      <c r="J13" s="6" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="5" t="inlineStr">
+        <is>
+          <t>tr_013</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="inlineStr">
+        <is>
+          <t>st_008</t>
+        </is>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>kauf</t>
+        </is>
+      </c>
+      <c r="D14" s="5" t="inlineStr">
+        <is>
+          <t>2025-10-03</t>
+        </is>
+      </c>
+      <c r="E14" s="5" t="n">
+        <v>28</v>
+      </c>
+      <c r="F14" s="5" t="n">
+        <v>572.4</v>
+      </c>
+      <c r="G14" s="5" t="inlineStr">
+        <is>
+          <t>SEK</t>
+        </is>
+      </c>
+      <c r="H14" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="I14" s="5" t="n">
+        <v>16027.2</v>
+      </c>
+      <c r="J14" s="5" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="6" t="inlineStr">
+        <is>
+          <t>tr_014</t>
+        </is>
+      </c>
+      <c r="B15" s="6" t="inlineStr">
+        <is>
+          <t>st_009</t>
+        </is>
+      </c>
+      <c r="C15" s="6" t="inlineStr">
+        <is>
+          <t>kauf</t>
+        </is>
+      </c>
+      <c r="D15" s="6" t="inlineStr">
+        <is>
+          <t>2026-01-14</t>
+        </is>
+      </c>
+      <c r="E15" s="6" t="n">
+        <v>11</v>
+      </c>
+      <c r="F15" s="6" t="n">
+        <v>60.2</v>
+      </c>
+      <c r="G15" s="6" t="inlineStr">
+        <is>
+          <t>CHF</t>
+        </is>
+      </c>
+      <c r="H15" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="I15" s="6" t="n">
+        <v>662.2</v>
+      </c>
+      <c r="J15" s="6" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="7" t="inlineStr">
+        <is>
+          <t>Typ: 'kauf' oder 'verkauf'  |  AktieID muss mit ID im Aktien-Sheet übereinstimmen</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
     <tabColor rgb="00888888"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>

</xml_diff>